<commit_message>
refactor: update session timeout duration, improve admin dashboard UI, and modernize WiFi naming page layout
</commit_message>
<xml_diff>
--- a/Modelos probados skypass.xlsx
+++ b/Modelos probados skypass.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/josemestre/Proyectos Jose/Sky Soluciones/skypass/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9465B868-F6E1-C845-9E6A-FBE99F5D3999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB487915-3449-1740-AFF9-375E024E9141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{EA3742AE-3201-0F48-9201-28932A5A462B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5091" uniqueCount="2322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5093" uniqueCount="2322">
   <si>
     <t>FD512XW-X-R330</t>
   </si>
@@ -7496,6 +7496,9 @@
       <c r="E10" t="s">
         <v>2320</v>
       </c>
+      <c r="F10" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="3:6" ht="18" x14ac:dyDescent="0.2">
       <c r="C11" s="1" t="s">
@@ -7549,6 +7552,9 @@
       </c>
       <c r="E16" t="s">
         <v>2320</v>
+      </c>
+      <c r="F16" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="3:4" ht="18" x14ac:dyDescent="0.2">

</xml_diff>